<commit_message>
Version 1.0 de ecosistema ETL
</commit_message>
<xml_diff>
--- a/proyecto_retail_etl/bodega_datos/1_brutos/metas_anuales.xlsx
+++ b/proyecto_retail_etl/bodega_datos/1_brutos/metas_anuales.xlsx
@@ -445,14 +445,14 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>913415</v>
+        <v>857088</v>
       </c>
       <c r="C2" t="n">
-        <v>12.04</v>
+        <v>11.06</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Tecnología</t>
+          <t>Deportes</t>
         </is>
       </c>
     </row>
@@ -463,14 +463,14 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1234596</v>
+        <v>2344238</v>
       </c>
       <c r="C3" t="n">
-        <v>6.73</v>
+        <v>17.17</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Tecnología</t>
+          <t>Moda</t>
         </is>
       </c>
     </row>
@@ -481,10 +481,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1387684</v>
+        <v>1155591</v>
       </c>
       <c r="C4" t="n">
-        <v>17.87</v>
+        <v>19.88</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -499,14 +499,14 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2487300</v>
+        <v>1652970</v>
       </c>
       <c r="C5" t="n">
-        <v>20.69</v>
+        <v>20.33</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Tecnología</t>
+          <t>Hogar</t>
         </is>
       </c>
     </row>
@@ -517,14 +517,14 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2450366</v>
+        <v>1199652</v>
       </c>
       <c r="C6" t="n">
-        <v>9.06</v>
+        <v>21.98</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Hogar</t>
+          <t>Tecnología</t>
         </is>
       </c>
     </row>
@@ -535,14 +535,14 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2241548</v>
+        <v>2468267</v>
       </c>
       <c r="C7" t="n">
-        <v>11.63</v>
+        <v>13.19</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Tecnología</t>
+          <t>Hogar</t>
         </is>
       </c>
     </row>
@@ -553,10 +553,10 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1440354</v>
+        <v>586142</v>
       </c>
       <c r="C8" t="n">
-        <v>7.78</v>
+        <v>21.64</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -571,14 +571,14 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1707309</v>
+        <v>795042</v>
       </c>
       <c r="C9" t="n">
-        <v>21.24</v>
+        <v>15.66</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Hogar</t>
+          <t>Deportes</t>
         </is>
       </c>
     </row>

</xml_diff>